<commit_message>
Latest publication got DOI, issue, etc)
</commit_message>
<xml_diff>
--- a/Data/marsja_publications.xlsx
+++ b/Data/marsja_publications.xlsx
@@ -1,46 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erima96\Dropbox\BetweenComps\Forskning\CV\Data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD68C0C4-0D13-48D2-A76C-787C208C106C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="publications" sheetId="1" r:id="rId1"/>
-    <sheet name="manuscripts" sheetId="2" r:id="rId2"/>
-    <sheet name="conferences" sheetId="3" r:id="rId3"/>
-    <sheet name="grants" sheetId="5" r:id="rId4"/>
-    <sheet name="peer_reviews" sheetId="6" r:id="rId5"/>
+    <sheet name="publications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="manuscripts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="conferences" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="grants" sheetId="5" state="visible" r:id="rId4"/>
+    <sheet name="peer_reviews" sheetId="6" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
   <si>
     <t>authors</t>
   </si>
@@ -910,6 +887,18 @@
   </si>
   <si>
     <t>Trends in Hearing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016/j.jth.2026.102454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102454</t>
   </si>
 </sst>
 </file>
@@ -919,7 +908,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0\ &quot;SEK&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -928,18 +917,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <b/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Carlito"/>
     </font>
     <font>
       <sz val="10"/>
@@ -979,31 +965,30 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF17365D"/>
       </left>
-      <right/>
       <top style="thin">
         <color rgb="FF17365D"/>
       </top>
       <bottom style="thin">
         <color rgb="FF17365D"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FF17365D"/>
       </top>
       <bottom style="thin">
         <color rgb="FF17365D"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FF17365D"/>
       </right>
@@ -1013,32 +998,17 @@
       <bottom style="thin">
         <color rgb="FF17365D"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD9E2F3"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color rgb="FF1F4E78"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1049,75 +1019,66 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{9A001293-7B37-43B1-A235-F7092CA9E873}"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
@@ -1269,6 +1230,16 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
+    <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+      <xfpb:xfComplement i="0"/>
+    </ext>
+  </extLst>
+  <extLst>
+    <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+      <xfpb:DXFComplement i="0"/>
+    </ext>
+  </extLst>
+  <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
@@ -1279,30 +1250,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3D94CBB8-7DE9-4243-8BAE-23F1DA2A9AF1}" name="PublicationsTable" displayName="PublicationsTable" ref="A1:K20" totalsRowShown="0">
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D94CBB8-7DE9-4243-8BAE-23F1DA2A9AF1}" name="PublicationsTable" displayName="PublicationsTable" ref="A1:K20" totalsRowShown="0">
   <autoFilter ref="A1:K20" xr:uid="{3D94CBB8-7DE9-4243-8BAE-23F1DA2A9AF1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K20">
     <sortCondition ref="E1:E20"/>
@@ -1324,8 +1273,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{438ADACE-1D0A-41AB-ADB3-11082AF927A1}" name="ManuscriptsTable" displayName="ManuscriptsTable" ref="A1:G10" totalsRowShown="0">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{438ADACE-1D0A-41AB-ADB3-11082AF927A1}" name="ManuscriptsTable" displayName="ManuscriptsTable" ref="A1:G10" totalsRowShown="0">
   <autoFilter ref="A1:G10" xr:uid="{438ADACE-1D0A-41AB-ADB3-11082AF927A1}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{BE401577-A3CF-40CB-AAF0-98A84EB859FD}" name="authors" dataDxfId="7"/>
@@ -1602,11 +1551,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1641,7 +1590,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1654,7 +1603,7 @@
       <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>2014</v>
       </c>
       <c r="F2" t="s">
@@ -1670,7 +1619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1683,7 +1632,7 @@
       <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>2018</v>
       </c>
       <c r="F3" t="s">
@@ -1705,7 +1654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1718,7 +1667,7 @@
       <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>2019</v>
       </c>
       <c r="F4" t="s">
@@ -1734,7 +1683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1747,7 +1696,7 @@
       <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>2020</v>
       </c>
       <c r="F5" t="s">
@@ -1766,7 +1715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1779,7 +1728,7 @@
       <c r="D6" t="s">
         <v>14</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>2021</v>
       </c>
       <c r="F6" t="s">
@@ -1798,7 +1747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1811,7 +1760,7 @@
       <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>2022</v>
       </c>
       <c r="F7" t="s">
@@ -1833,7 +1782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1846,7 +1795,7 @@
       <c r="D8" t="s">
         <v>14</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>2022</v>
       </c>
       <c r="F8" t="s">
@@ -1868,7 +1817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -1881,7 +1830,7 @@
       <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>2023</v>
       </c>
       <c r="F9" t="s">
@@ -1903,7 +1852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -1916,7 +1865,7 @@
       <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>2024</v>
       </c>
       <c r="F10" t="s">
@@ -1938,7 +1887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1951,7 +1900,7 @@
       <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>2024</v>
       </c>
       <c r="F11" t="s">
@@ -1973,7 +1922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -1986,7 +1935,7 @@
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>2025</v>
       </c>
       <c r="F12" t="s">
@@ -2005,7 +1954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -2018,7 +1967,7 @@
       <c r="D13" t="s">
         <v>14</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
@@ -2037,7 +1986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2050,7 +1999,7 @@
       <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>2025</v>
       </c>
       <c r="F14" t="s">
@@ -2072,7 +2021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15">
       <c r="A15" t="s">
         <v>95</v>
       </c>
@@ -2085,7 +2034,7 @@
       <c r="D15" t="s">
         <v>14</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>2026</v>
       </c>
       <c r="F15" t="s">
@@ -2104,7 +2053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16">
       <c r="A16" t="s">
         <v>102</v>
       </c>
@@ -2117,7 +2066,7 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>2026</v>
       </c>
       <c r="F16" t="s">
@@ -2139,7 +2088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17">
       <c r="A17" t="s">
         <v>108</v>
       </c>
@@ -2152,7 +2101,7 @@
       <c r="D17" t="s">
         <v>14</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>2026</v>
       </c>
       <c r="F17" t="s">
@@ -2174,7 +2123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18">
       <c r="A18" t="s">
         <v>113</v>
       </c>
@@ -2209,7 +2158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19">
       <c r="A19" t="s">
         <v>108</v>
       </c>
@@ -2226,7 +2175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20">
       <c r="A20" t="s">
         <v>123</v>
       </c>
@@ -2238,6 +2187,18 @@
       </c>
       <c r="D20" t="s">
         <v>116</v>
+      </c>
+      <c r="E20" t="s">
+        <v>291</v>
+      </c>
+      <c r="F20" t="s">
+        <v>292</v>
+      </c>
+      <c r="H20" t="s">
+        <v>293</v>
+      </c>
+      <c r="I20" t="s">
+        <v>290</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -2256,21 +2217,22 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6762FCB3-B13D-4734-9F5E-9E8B06F6555F}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="3" max="3" width="98.42578125" customWidth="1"/>
+    <col min="3" max="3" width="98.42578125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="25.5">
+    <row r="1" ht="25.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2293,7 +2255,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="165.75">
+    <row r="2" ht="165.75" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>129</v>
       </c>
@@ -2303,16 +2265,16 @@
       <c r="C2" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D2" s="4" t="b">
+      <c r="D2" s="3" t="b">
         <v>1</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="4" t="b">
+      <c r="F2" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="255">
+    <row r="3" ht="255" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>132</v>
       </c>
@@ -2322,16 +2284,16 @@
       <c r="C3" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D3" s="4" t="b">
+      <c r="D3" s="3" t="b">
         <v>1</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="4" t="b">
+      <c r="F3" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="204">
+    <row r="4" ht="204" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>135</v>
       </c>
@@ -2341,16 +2303,16 @@
       <c r="C4" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="4" t="b">
+      <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E4" s="3"/>
-      <c r="F4" s="4" t="b">
+      <c r="F4" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="178.5">
+    <row r="5" ht="178.5" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>137</v>
       </c>
@@ -2360,16 +2322,16 @@
       <c r="C5" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="4" t="b">
+      <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E5" s="3"/>
-      <c r="F5" s="4" t="b">
+      <c r="F5" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="216.75">
+    <row r="6" ht="216.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>129</v>
       </c>
@@ -2379,16 +2341,16 @@
       <c r="C6" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D6" s="4" t="b">
+      <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="F6" s="4" t="b">
+      <c r="F6" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" ht="165.75">
+    <row r="7" ht="165.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>140</v>
       </c>
@@ -2398,16 +2360,16 @@
       <c r="C7" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="4" t="b">
+      <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="4" t="b">
+      <c r="F7" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" ht="216.75">
+    <row r="8" ht="216.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>142</v>
       </c>
@@ -2417,16 +2379,16 @@
       <c r="C8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D8" s="4" t="b">
+      <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="4" t="b">
+      <c r="F8" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="178.5">
+    <row r="9" ht="178.5" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>144</v>
       </c>
@@ -2436,16 +2398,16 @@
       <c r="C9" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="4" t="b">
+      <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E9" s="3"/>
-      <c r="F9" s="4" t="b">
+      <c r="F9" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="178.5">
+    <row r="10" ht="178.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>146</v>
       </c>
@@ -2455,13 +2417,13 @@
       <c r="C10" t="s">
         <v>148</v>
       </c>
-      <c r="D10" s="4" t="b">
+      <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
       <c r="E10" t="s">
         <v>149</v>
       </c>
-      <c r="F10" s="4" t="b">
+      <c r="F10" s="3" t="b">
         <v>1</v>
       </c>
       <c r="G10" s="2"/>
@@ -2481,1398 +2443,1402 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E423594E-FBE8-4DDC-98B2-E9633CC9D2B3}">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="38.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="38.25" customHeight="1">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="242.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" ht="242.25" customHeight="1">
+      <c r="A2" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="8" t="n">
         <v>2026</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="216.75">
-      <c r="A3" s="9" t="s">
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="216.75" customHeight="1">
+      <c r="A3" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="216.75">
-      <c r="A4" s="8" t="s">
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="216.75" customHeight="1">
+      <c r="A4" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="153">
-      <c r="A5" s="9" t="s">
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="153" customHeight="1">
+      <c r="A5" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="255">
-      <c r="A6" s="8" t="s">
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="255" customHeight="1">
+      <c r="A6" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="178.5">
-      <c r="A7" s="9" t="s">
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="178.5" customHeight="1">
+      <c r="A7" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="13" t="s">
+      <c r="F7" s="14"/>
+      <c r="G7" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="127.5">
-      <c r="A8" s="8" t="s">
+      <c r="J7" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="127.5" customHeight="1">
+      <c r="A8" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="8" t="n">
         <v>2024</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="89.25">
-      <c r="A9" s="9" t="s">
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="89.25" customHeight="1">
+      <c r="A9" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9" t="s">
+      <c r="H9" s="14"/>
+      <c r="I9" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="J9" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="216.75">
-      <c r="A10" s="8" t="s">
+      <c r="J9" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="216.75" customHeight="1">
+      <c r="A10" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="165.75">
-      <c r="A11" s="9" t="s">
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="165.75" customHeight="1">
+      <c r="A11" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="9" t="s">
+      <c r="D11" s="5"/>
+      <c r="E11" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="13" t="s">
+      <c r="F11" s="14"/>
+      <c r="G11" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="J11" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="178.5">
-      <c r="A12" s="8" t="s">
+      <c r="J11" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="178.5" customHeight="1">
+      <c r="A12" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="8" t="n">
         <v>2019</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="G12" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="178.5">
-      <c r="A13" s="9" t="s">
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="178.5" customHeight="1">
+      <c r="A13" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="9" t="n">
         <v>2019</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="127.5">
-      <c r="A14" s="8" t="s">
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="127.5" customHeight="1">
+      <c r="A14" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="8" t="n">
         <v>2019</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="140.25">
-      <c r="A15" s="9" t="s">
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="140.25" customHeight="1">
+      <c r="A15" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="9" t="n">
         <v>2019</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G15" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="140.25">
-      <c r="A16" s="8" t="s">
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="140.25" customHeight="1">
+      <c r="A16" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="8" t="n">
         <v>2019</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="178.5">
-      <c r="A17" s="9" t="s">
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="178.5" customHeight="1">
+      <c r="A17" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="9" t="n">
         <v>2017</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="191.25">
-      <c r="A18" s="8" t="s">
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" ht="191.25" customHeight="1">
+      <c r="A18" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="8" t="n">
         <v>2016</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8" t="s">
+      <c r="H18" s="13"/>
+      <c r="I18" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="J18" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="165.75">
-      <c r="A19" s="9" t="s">
+      <c r="J18" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" ht="165.75" customHeight="1">
+      <c r="A19" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="9" t="n">
         <v>2016</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="178.5">
-      <c r="A20" s="8" t="s">
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" ht="178.5" customHeight="1">
+      <c r="A20" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="8" t="n">
         <v>2015</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="140.25">
-      <c r="A21" s="9" t="s">
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" ht="140.25" customHeight="1">
+      <c r="A21" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="9" t="n">
         <v>2014</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="204">
-      <c r="A22" s="8" t="s">
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="204" customHeight="1">
+      <c r="A22" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="8" t="n">
         <v>2014</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="13" t="s">
         <v>235</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="G22" s="12" t="s">
+      <c r="G22" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="140.25">
-      <c r="A23" s="9" t="s">
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" ht="140.25" customHeight="1">
+      <c r="A23" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="9" t="n">
         <v>2013</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="G23" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="11" t="b">
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="5" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D875878-16C3-4B80-856A-BDFA6FCE6383}">
-  <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="25.5">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="25.5" customHeight="1">
+      <c r="A1" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="255">
-      <c r="A2" s="8" t="s">
+    <row r="2" ht="255" customHeight="1">
+      <c r="A2" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="15" t="n">
         <v>6000</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="16" t="n">
         <v>2013</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="F2" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="8"/>
-    </row>
-    <row r="3" spans="1:9" ht="127.5">
-      <c r="A3" s="9" t="s">
+      <c r="F2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="13"/>
+    </row>
+    <row r="3" ht="127.5" customHeight="1">
+      <c r="A3" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="B3" s="18">
+      <c r="B3" s="17" t="n">
         <v>10000</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="18" t="n">
         <v>2014</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="F3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="9"/>
-    </row>
-    <row r="4" spans="1:9" ht="216.75">
-      <c r="A4" s="8" t="s">
+      <c r="F3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="14"/>
+    </row>
+    <row r="4" ht="216.75" customHeight="1">
+      <c r="A4" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="15" t="n">
         <v>9000</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="16" t="n">
         <v>2014</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="F4" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9" ht="191.25">
-      <c r="A5" s="9" t="s">
+      <c r="F4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="13"/>
+    </row>
+    <row r="5" ht="191.25" customHeight="1">
+      <c r="A5" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="17" t="n">
         <v>15000</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="18" t="n">
         <v>2016</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="9"/>
-    </row>
-    <row r="6" spans="1:9" ht="255">
-      <c r="A6" s="8" t="s">
+      <c r="F5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="14"/>
+    </row>
+    <row r="6" ht="255" customHeight="1">
+      <c r="A6" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15" t="n">
         <v>12000</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16" t="n">
         <v>2016</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="13" t="s">
         <v>257</v>
       </c>
-      <c r="F6" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="8"/>
-    </row>
-    <row r="7" spans="1:9" ht="165.75">
-      <c r="A7" s="9" t="s">
+      <c r="F6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="13"/>
+    </row>
+    <row r="7" ht="165.75" customHeight="1">
+      <c r="A7" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="17" t="n">
         <v>8000</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="18" t="n">
         <v>2016</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="F7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="9"/>
-    </row>
-    <row r="8" spans="1:9" ht="127.5">
-      <c r="A8" s="8" t="s">
+      <c r="F7" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="14"/>
+    </row>
+    <row r="8" ht="127.5" customHeight="1">
+      <c r="A8" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15" t="n">
         <v>6000</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="16" t="n">
         <v>2017</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="F8" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="8"/>
-    </row>
-    <row r="9" spans="1:9" ht="318.75">
-      <c r="A9" s="9" t="s">
+      <c r="F8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="13"/>
+    </row>
+    <row r="9" ht="318.75" customHeight="1">
+      <c r="A9" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="17" t="n">
         <v>299235</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="18" t="n">
         <v>2021</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="F9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="9"/>
-    </row>
-    <row r="10" spans="1:9" ht="140.25">
-      <c r="A10" s="8" t="s">
+      <c r="F9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="14"/>
+    </row>
+    <row r="10" ht="140.25" customHeight="1">
+      <c r="A10" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15" t="n">
         <v>4170000</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="16" t="n">
         <v>2023</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="F10" s="10" t="b">
+      <c r="F10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="8" t="s">
+      <c r="G10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="13" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="382.5">
-      <c r="A11" s="9" t="s">
+    <row r="11" ht="382.5" customHeight="1">
+      <c r="A11" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="17" t="n">
         <v>3391904</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="18" t="n">
         <v>2025</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="F11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="9"/>
-    </row>
-    <row r="12" spans="1:9" ht="140.25">
-      <c r="A12" s="8" t="s">
+      <c r="F11" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="14"/>
+    </row>
+    <row r="12" ht="140.25" customHeight="1">
+      <c r="A12" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15" t="n">
         <v>103600</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="16" t="n">
         <v>2026</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="13" t="s">
         <v>269</v>
       </c>
-      <c r="F12" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="8"/>
+      <c r="F12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB5DDDD8-49F9-4998-AC22-6C371210FCFB}">
-  <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A1" s="20" t="s">
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="19" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="21" t="s">
+    <row r="2">
+      <c r="A2" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="21" t="n">
         <v>2018</v>
       </c>
-      <c r="C2" s="22">
-        <v>1</v>
-      </c>
-      <c r="D2" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="21" t="s">
+      <c r="C2" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="21" t="n">
         <v>2022</v>
       </c>
-      <c r="C3" s="22">
-        <v>1</v>
-      </c>
-      <c r="D3" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="21" t="s">
+      <c r="C3" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="C4" s="22">
-        <v>1</v>
-      </c>
-      <c r="D4" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="21" t="s">
+      <c r="C4" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="C5" s="22">
-        <v>1</v>
-      </c>
-      <c r="D5" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="21" t="s">
+      <c r="C5" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="C6" s="22">
-        <v>1</v>
-      </c>
-      <c r="D6" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="21" t="s">
+      <c r="C6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="21" t="n">
         <v>2024</v>
       </c>
-      <c r="C7" s="22">
-        <v>1</v>
-      </c>
-      <c r="D7" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="21" t="s">
+      <c r="C7" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="21" t="n">
         <v>2024</v>
       </c>
-      <c r="C8" s="22">
-        <v>1</v>
-      </c>
-      <c r="D8" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="21" t="s">
+      <c r="C8" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="21" t="n">
         <v>2024</v>
       </c>
-      <c r="C9" s="22">
-        <v>1</v>
-      </c>
-      <c r="D9" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="21" t="s">
+      <c r="C9" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C10" s="22">
-        <v>1</v>
-      </c>
-      <c r="D10" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="21" t="s">
+      <c r="C10" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C11" s="22">
-        <v>1</v>
-      </c>
-      <c r="D11" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="21" t="s">
+      <c r="C11" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C12" s="22">
-        <v>1</v>
-      </c>
-      <c r="D12" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="21" t="s">
+      <c r="C12" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="s">
         <v>278</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C13" s="22">
-        <v>1</v>
-      </c>
-      <c r="D13" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="21" t="s">
+      <c r="C13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C14" s="22">
-        <v>1</v>
-      </c>
-      <c r="D14" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="21" t="s">
+      <c r="C14" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="C15" s="22">
-        <v>1</v>
-      </c>
-      <c r="D15" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="21" t="s">
+      <c r="C15" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C16" s="22">
-        <v>1</v>
-      </c>
-      <c r="D16" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="21" t="s">
+      <c r="C16" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="B17" s="22">
+      <c r="B17" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C17" s="22">
-        <v>1</v>
-      </c>
-      <c r="D17" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="21" t="s">
+      <c r="C17" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="s">
         <v>283</v>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C18" s="22">
-        <v>1</v>
-      </c>
-      <c r="D18" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="21" t="s">
+      <c r="C18" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="B19" s="22">
+      <c r="B19" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C19" s="22">
-        <v>1</v>
-      </c>
-      <c r="D19" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="21" t="s">
+      <c r="C19" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C20" s="22">
-        <v>1</v>
-      </c>
-      <c r="D20" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="21" t="s">
+      <c r="C20" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C21" s="22">
-        <v>1</v>
-      </c>
-      <c r="D21" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="21" t="s">
+      <c r="C21" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C22" s="22">
-        <v>1</v>
-      </c>
-      <c r="D22" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="21" t="s">
+      <c r="C22" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C23" s="22">
-        <v>1</v>
-      </c>
-      <c r="D23" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="21" t="s">
+      <c r="C23" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="s">
         <v>287</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C24" s="22">
-        <v>1</v>
-      </c>
-      <c r="D24" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="21" t="s">
+      <c r="C24" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C25" s="22">
-        <v>1</v>
-      </c>
-      <c r="D25" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="21" t="s">
+      <c r="C25" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="s">
         <v>278</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C26" s="22">
-        <v>1</v>
-      </c>
-      <c r="D26" s="23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="21" t="s">
+      <c r="C26" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C27" s="22">
-        <v>1</v>
-      </c>
-      <c r="D27" s="23" t="b">
+      <c r="C27" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="22" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated CV, added link to publikation
</commit_message>
<xml_diff>
--- a/Data/marsja_publications.xlsx
+++ b/Data/marsja_publications.xlsx
@@ -1,23 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erima96\Dropbox\BetweenComps\Forskning\CV\Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2AD1E030-C0BE-4A48-A096-AF0770B9EDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="0" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="publications" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="manuscripts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="conferences" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="grants" sheetId="5" state="visible" r:id="rId4"/>
-    <sheet name="peer_reviews" sheetId="6" state="visible" r:id="rId5"/>
+    <sheet name="publications" sheetId="1" r:id="rId1"/>
+    <sheet name="manuscripts" sheetId="2" r:id="rId2"/>
+    <sheet name="conferences" sheetId="3" r:id="rId3"/>
+    <sheet name="grants" sheetId="5" r:id="rId4"/>
+    <sheet name="peer_reviews" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="295">
   <si>
     <t>authors</t>
   </si>
@@ -889,26 +897,26 @@
     <t>Trends in Hearing</t>
   </si>
   <si>
-    <t xml:space="preserve">10.1016/j.jth.2026.102454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52</t>
-  </si>
-  <si>
-    <t xml:space="preserve">102454</t>
+    <t>10.1016/j.jth.2026.102454</t>
+  </si>
+  <si>
+    <t>2027</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>102454</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Ec9miqeO2wU7uOoXzluMigdVlJJYZLVf/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0\ &quot;SEK&quot;"/>
-  </numFmts>
-  <fonts count="5">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -917,28 +925,134 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF222222"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -947,16 +1061,179 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4F7FB"/>
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -965,280 +1242,206 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin">
-        <color rgb="FFD9E2F3"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FF7F7F7F"/>
       </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
       <top style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FF7F7F7F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FF7F7F7F"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
       <right style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FFB2B2B2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF17365D"/>
+        <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
-      <bottom style="medium">
-        <color rgb="FF1F4E78"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="42">
+    <cellStyle name="20 % - Dekorfärg1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20 % - Dekorfärg2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20 % - Dekorfärg3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20 % - Dekorfärg4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20 % - Dekorfärg5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20 % - Dekorfärg6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40 % - Dekorfärg6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60 % - Dekorfärg6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Anteckning" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Beräkning" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Bra" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Dekorfärg6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Dålig" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Förklarande text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Indata" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Kontrollcell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Länkad cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Rubrik" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Rubrik 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Rubrik 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Rubrik 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Rubrik 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Summa" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Utdata" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Varningstext" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <font>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-      <xfpb:xfComplement i="0"/>
-    </ext>
-  </extLst>
-  <extLst>
-    <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-      <xfpb:DXFComplement i="0"/>
-    </ext>
-  </extLst>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1250,7 +1453,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D94CBB8-7DE9-4243-8BAE-23F1DA2A9AF1}" name="PublicationsTable" displayName="PublicationsTable" ref="A1:K20" totalsRowShown="0">
   <autoFilter ref="A1:K20" xr:uid="{3D94CBB8-7DE9-4243-8BAE-23F1DA2A9AF1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K20">
@@ -1273,17 +1476,17 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{438ADACE-1D0A-41AB-ADB3-11082AF927A1}" name="ManuscriptsTable" displayName="ManuscriptsTable" ref="A1:G10" totalsRowShown="0">
   <autoFilter ref="A1:G10" xr:uid="{438ADACE-1D0A-41AB-ADB3-11082AF927A1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BE401577-A3CF-40CB-AAF0-98A84EB859FD}" name="authors" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{18DD88C4-63C3-469F-B983-59A217450048}" name="title" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{4FB386F2-5B3C-4445-B094-808E28C68A26}" name="status" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{BC683C7A-D801-409C-B703-633910D5349A}" name="double_blind" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{E88FE722-D6F6-4DAD-88A0-3D14BB2071D0}" name="url" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{ED27018D-E416-41A3-B654-E9A2CBAD566E}" name="include_cv" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{A4E57606-FCFF-458F-A87D-8F6B14F26BCA}" name="notes" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{BE401577-A3CF-40CB-AAF0-98A84EB859FD}" name="authors"/>
+    <tableColumn id="2" xr3:uid="{18DD88C4-63C3-469F-B983-59A217450048}" name="title"/>
+    <tableColumn id="3" xr3:uid="{4FB386F2-5B3C-4445-B094-808E28C68A26}" name="status"/>
+    <tableColumn id="4" xr3:uid="{BC683C7A-D801-409C-B703-633910D5349A}" name="double_blind"/>
+    <tableColumn id="5" xr3:uid="{E88FE722-D6F6-4DAD-88A0-3D14BB2071D0}" name="url"/>
+    <tableColumn id="6" xr3:uid="{ED27018D-E416-41A3-B654-E9A2CBAD566E}" name="include_cv"/>
+    <tableColumn id="7" xr3:uid="{A4E57606-FCFF-458F-A87D-8F6B14F26BCA}" name="notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1551,11 +1754,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1590,7 +1793,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1603,7 +1806,7 @@
       <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>2014</v>
       </c>
       <c r="F2" t="s">
@@ -1619,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1632,7 +1835,7 @@
       <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>2018</v>
       </c>
       <c r="F3" t="s">
@@ -1654,7 +1857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1667,7 +1870,7 @@
       <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>2019</v>
       </c>
       <c r="F4" t="s">
@@ -1683,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1696,7 +1899,7 @@
       <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>2020</v>
       </c>
       <c r="F5" t="s">
@@ -1715,7 +1918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1728,7 +1931,7 @@
       <c r="D6" t="s">
         <v>14</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>2021</v>
       </c>
       <c r="F6" t="s">
@@ -1747,7 +1950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1760,7 +1963,7 @@
       <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>2022</v>
       </c>
       <c r="F7" t="s">
@@ -1782,7 +1985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1795,7 +1998,7 @@
       <c r="D8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>2022</v>
       </c>
       <c r="F8" t="s">
@@ -1817,7 +2020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -1830,7 +2033,7 @@
       <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>2023</v>
       </c>
       <c r="F9" t="s">
@@ -1852,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -1865,7 +2068,7 @@
       <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>2024</v>
       </c>
       <c r="F10" t="s">
@@ -1887,7 +2090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1900,7 +2103,7 @@
       <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>2024</v>
       </c>
       <c r="F11" t="s">
@@ -1922,7 +2125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -1935,7 +2138,7 @@
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>2025</v>
       </c>
       <c r="F12" t="s">
@@ -1954,7 +2157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -1967,7 +2170,7 @@
       <c r="D13" t="s">
         <v>14</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
@@ -1986,7 +2189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -1999,7 +2202,7 @@
       <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" t="s">
@@ -2021,7 +2224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>95</v>
       </c>
@@ -2034,7 +2237,7 @@
       <c r="D15" t="s">
         <v>14</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>2026</v>
       </c>
       <c r="F15" t="s">
@@ -2053,7 +2256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>102</v>
       </c>
@@ -2066,7 +2269,7 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>2026</v>
       </c>
       <c r="F16" t="s">
@@ -2088,7 +2291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>108</v>
       </c>
@@ -2101,7 +2304,7 @@
       <c r="D17" t="s">
         <v>14</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>2026</v>
       </c>
       <c r="F17" t="s">
@@ -2123,7 +2326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>113</v>
       </c>
@@ -2158,7 +2361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>108</v>
       </c>
@@ -2175,7 +2378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>123</v>
       </c>
@@ -2199,6 +2402,9 @@
       </c>
       <c r="I20" t="s">
         <v>290</v>
+      </c>
+      <c r="J20" t="s">
+        <v>294</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -2217,220 +2423,203 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="98.42578125" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="98.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>126</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>127</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" ht="165.75" customHeight="1">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:7" ht="165.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>130</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>131</v>
       </c>
-      <c r="D2" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" ht="255" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="255" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>134</v>
       </c>
-      <c r="D3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" ht="204" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="204" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="3" t="b">
+      <c r="D4" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" ht="178.5" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>137</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>138</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="3" t="b">
+      <c r="D5" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" ht="216.75" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>139</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>131</v>
       </c>
-      <c r="D6" s="3" t="b">
+      <c r="D6" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" ht="165.75" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="165.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>131</v>
       </c>
-      <c r="D7" s="3" t="b">
+      <c r="D7" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" ht="216.75" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>142</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" t="s">
         <v>131</v>
       </c>
-      <c r="D8" s="3" t="b">
+      <c r="D8" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" ht="178.5" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>144</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>145</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="3" t="b">
+      <c r="D9" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" ht="178.5" customHeight="1">
-      <c r="A10" s="2" t="s">
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>146</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>147</v>
       </c>
       <c r="C10" t="s">
         <v>148</v>
       </c>
-      <c r="D10" s="3" t="b">
+      <c r="D10" t="b">
         <v>0</v>
       </c>
       <c r="E10" t="s">
         <v>149</v>
       </c>
-      <c r="F10" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" s="2"/>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:G9 A10:B10 D10:G10">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" priority="1">
       <formula>$D2=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2443,1402 +2632,1351 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="38.25" customHeight="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:10" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" t="s">
         <v>150</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" t="s">
         <v>151</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" t="s">
         <v>152</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" t="s">
         <v>153</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" t="s">
         <v>127</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" t="s">
         <v>128</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="242.25" customHeight="1">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:10" ht="242.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>154</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2">
         <v>2026</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" t="s">
         <v>156</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" t="s">
         <v>157</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" t="s">
         <v>158</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" t="s">
         <v>159</v>
       </c>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" ht="216.75" customHeight="1">
-      <c r="A3" s="14" t="s">
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3">
         <v>2025</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" t="s">
         <v>156</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" t="s">
         <v>162</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" t="s">
         <v>163</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="216.75" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" t="s">
         <v>165</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4">
         <v>2025</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" t="s">
         <v>167</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" t="s">
         <v>168</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" t="s">
         <v>169</v>
       </c>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" ht="153" customHeight="1">
-      <c r="A5" s="14" t="s">
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="153" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" t="s">
         <v>170</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5">
         <v>2025</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" t="s">
         <v>166</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" t="s">
         <v>167</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" t="s">
         <v>168</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" t="s">
         <v>169</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="255" customHeight="1">
-      <c r="A6" s="13" t="s">
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="255" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>171</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6">
         <v>2025</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" t="s">
         <v>166</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" t="s">
         <v>167</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" t="s">
         <v>168</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" t="s">
         <v>169</v>
       </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" ht="178.5" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7">
         <v>2024</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" t="s">
         <v>175</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" t="s">
         <v>176</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="7" t="s">
+      <c r="G7" t="s">
         <v>169</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" t="s">
         <v>177</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" ht="127.5" customHeight="1">
-      <c r="A8" s="13" t="s">
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>179</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" t="s">
         <v>180</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8">
         <v>2024</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" t="s">
         <v>166</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" t="s">
         <v>167</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" t="s">
         <v>181</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" t="s">
         <v>169</v>
       </c>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" ht="89.25" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>182</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" t="s">
         <v>183</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9">
         <v>2024</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" t="s">
         <v>167</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14" t="s">
+      <c r="I9" t="s">
         <v>184</v>
       </c>
-      <c r="J9" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="216.75" customHeight="1">
-      <c r="A10" s="13" t="s">
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" t="s">
         <v>186</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10">
         <v>2023</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" t="s">
         <v>188</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" t="s">
         <v>189</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" t="s">
         <v>169</v>
       </c>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" ht="165.75" customHeight="1">
-      <c r="A11" s="14" t="s">
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="165.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>190</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" t="s">
         <v>191</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11">
         <v>2023</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="14" t="s">
+      <c r="E11" t="s">
         <v>192</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="7" t="s">
+      <c r="G11" t="s">
         <v>193</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" t="s">
         <v>194</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" t="s">
         <v>195</v>
       </c>
-      <c r="J11" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="178.5" customHeight="1">
-      <c r="A12" s="13" t="s">
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>196</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12">
         <v>2019</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" t="s">
         <v>198</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" t="s">
         <v>199</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" t="s">
         <v>200</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="178.5" customHeight="1">
-      <c r="A13" s="14" t="s">
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>201</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" t="s">
         <v>202</v>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13">
         <v>2019</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" t="s">
         <v>200</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" t="s">
         <v>169</v>
       </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="127.5" customHeight="1">
-      <c r="A14" s="13" t="s">
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>203</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" t="s">
         <v>204</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14">
         <v>2019</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" t="s">
         <v>198</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" t="s">
         <v>205</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" t="s">
         <v>206</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" t="s">
         <v>169</v>
       </c>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="140.25" customHeight="1">
-      <c r="A15" s="14" t="s">
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>196</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" t="s">
         <v>207</v>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15">
         <v>2019</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" t="s">
         <v>156</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" t="s">
         <v>208</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" t="s">
         <v>209</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" t="s">
         <v>169</v>
       </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="140.25" customHeight="1">
-      <c r="A16" s="13" t="s">
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>210</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" t="s">
         <v>211</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16">
         <v>2019</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" t="s">
         <v>156</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" t="s">
         <v>208</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" t="s">
         <v>209</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" t="s">
         <v>169</v>
       </c>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" ht="178.5" customHeight="1">
-      <c r="A17" s="14" t="s">
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>212</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" t="s">
         <v>213</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17">
         <v>2017</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" t="s">
         <v>214</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E17" t="s">
         <v>215</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" t="s">
         <v>216</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" t="s">
         <v>169</v>
       </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" ht="191.25" customHeight="1">
-      <c r="A18" s="13" t="s">
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>212</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" t="s">
         <v>217</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18">
         <v>2016</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" t="s">
         <v>218</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" t="s">
         <v>219</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" t="s">
         <v>220</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13" t="s">
+      <c r="I18" t="s">
         <v>221</v>
       </c>
-      <c r="J18" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" ht="165.75" customHeight="1">
-      <c r="A19" s="14" t="s">
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="165.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>212</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" t="s">
         <v>222</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19">
         <v>2016</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" t="s">
         <v>156</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" t="s">
         <v>223</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" t="s">
         <v>224</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" t="s">
         <v>159</v>
       </c>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" ht="178.5" customHeight="1">
-      <c r="A20" s="13" t="s">
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>225</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" t="s">
         <v>226</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20">
         <v>2015</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" t="s">
         <v>187</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" t="s">
         <v>227</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="F20" t="s">
         <v>228</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" t="s">
         <v>169</v>
       </c>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" ht="140.25" customHeight="1">
-      <c r="A21" s="14" t="s">
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>229</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" t="s">
         <v>230</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21">
         <v>2014</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" t="s">
         <v>175</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" t="s">
         <v>231</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" t="s">
         <v>232</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" t="s">
         <v>169</v>
       </c>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" ht="204" customHeight="1">
-      <c r="A22" s="13" t="s">
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="204" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>233</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" t="s">
         <v>234</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22">
         <v>2014</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" t="s">
         <v>166</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" t="s">
         <v>235</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" t="s">
         <v>236</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" t="s">
         <v>169</v>
       </c>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" ht="140.25" customHeight="1">
-      <c r="A23" s="14" t="s">
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>229</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" t="s">
         <v>237</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23">
         <v>2013</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" t="s">
         <v>175</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" t="s">
         <v>238</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="F23" t="s">
         <v>239</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" t="s">
         <v>169</v>
       </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="5" t="b">
+      <c r="J23" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" t="s">
         <v>241</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" t="s">
         <v>242</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" t="s">
         <v>243</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" t="s">
         <v>244</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" t="s">
         <v>245</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" ht="255" customHeight="1">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:9" ht="255" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>246</v>
       </c>
-      <c r="B2" s="15" t="n">
+      <c r="B2">
         <v>6000</v>
       </c>
-      <c r="C2" s="16" t="n">
+      <c r="C2">
         <v>2013</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" t="s">
         <v>247</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" t="s">
         <v>248</v>
       </c>
-      <c r="F2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="13"/>
-    </row>
-    <row r="3" ht="127.5" customHeight="1">
-      <c r="A3" s="14" t="s">
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>249</v>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3">
         <v>10000</v>
       </c>
-      <c r="C3" s="18" t="n">
+      <c r="C3">
         <v>2014</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" t="s">
         <v>250</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" t="s">
         <v>251</v>
       </c>
-      <c r="F3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="14"/>
-    </row>
-    <row r="4" ht="216.75" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>252</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4">
         <v>9000</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4">
         <v>2014</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" t="s">
         <v>247</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" t="s">
         <v>253</v>
       </c>
-      <c r="F4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" ht="191.25" customHeight="1">
-      <c r="A5" s="14" t="s">
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>254</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5">
         <v>15000</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5">
         <v>2016</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" t="s">
         <v>250</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="14"/>
-    </row>
-    <row r="6" ht="255" customHeight="1">
-      <c r="A6" s="13" t="s">
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="255" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>256</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6">
         <v>12000</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6">
         <v>2016</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" t="s">
         <v>247</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" t="s">
         <v>257</v>
       </c>
-      <c r="F6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="13"/>
-    </row>
-    <row r="7" ht="165.75" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="165.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>246</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7">
         <v>8000</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7">
         <v>2016</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>247</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" t="s">
         <v>258</v>
       </c>
-      <c r="F7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="14"/>
-    </row>
-    <row r="8" ht="127.5" customHeight="1">
-      <c r="A8" s="13" t="s">
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8">
         <v>6000</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8">
         <v>2017</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" t="s">
         <v>247</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" t="s">
         <v>259</v>
       </c>
-      <c r="F8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9" ht="318.75" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="318.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>260</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9">
         <v>299235</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9">
         <v>2021</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" t="s">
         <v>250</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" t="s">
         <v>261</v>
       </c>
-      <c r="F9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="14"/>
-    </row>
-    <row r="10" ht="140.25" customHeight="1">
-      <c r="A10" s="13" t="s">
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>262</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10">
         <v>4170000</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10">
         <v>2023</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" t="s">
         <v>250</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" t="s">
         <v>263</v>
       </c>
-      <c r="F10" s="4" t="b">
+      <c r="F10" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="13" t="s">
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="11" ht="382.5" customHeight="1">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:9" ht="382.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>265</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11">
         <v>3391904</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11">
         <v>2025</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" t="s">
         <v>250</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" t="s">
         <v>266</v>
       </c>
-      <c r="F11" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="14"/>
-    </row>
-    <row r="12" ht="140.25" customHeight="1">
-      <c r="A12" s="13" t="s">
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>267</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12">
         <v>103600</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12">
         <v>2026</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" t="s">
         <v>268</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" t="s">
         <v>269</v>
       </c>
-      <c r="F12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" s="13"/>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" t="s">
         <v>270</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="20" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="21" t="n">
+      <c r="B2">
         <v>2018</v>
       </c>
-      <c r="C2" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="20" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>271</v>
       </c>
-      <c r="B3" s="21" t="n">
+      <c r="B3">
         <v>2022</v>
       </c>
-      <c r="C3" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="20" t="s">
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>272</v>
       </c>
-      <c r="B4" s="21" t="n">
+      <c r="B4">
         <v>2023</v>
       </c>
-      <c r="C4" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="20" t="s">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5">
         <v>2023</v>
       </c>
-      <c r="C5" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="20" t="s">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>271</v>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6">
         <v>2023</v>
       </c>
-      <c r="C6" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="20" t="s">
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>273</v>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7">
         <v>2024</v>
       </c>
-      <c r="C7" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="s">
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8">
         <v>2024</v>
       </c>
-      <c r="C8" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="20" t="s">
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>274</v>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9">
         <v>2024</v>
       </c>
-      <c r="C9" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="s">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>275</v>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10">
         <v>2025</v>
       </c>
-      <c r="C10" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="s">
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>276</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11">
         <v>2025</v>
       </c>
-      <c r="C11" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="s">
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>277</v>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12">
         <v>2025</v>
       </c>
-      <c r="C12" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="s">
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>278</v>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13">
         <v>2025</v>
       </c>
-      <c r="C13" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="s">
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>279</v>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14">
         <v>2025</v>
       </c>
-      <c r="C14" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="s">
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>280</v>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15">
         <v>2025</v>
       </c>
-      <c r="C15" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="s">
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16">
         <v>2026</v>
       </c>
-      <c r="C16" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="20" t="s">
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>282</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17">
         <v>2026</v>
       </c>
-      <c r="C17" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="s">
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>283</v>
       </c>
-      <c r="B18" s="21" t="n">
+      <c r="B18">
         <v>2026</v>
       </c>
-      <c r="C18" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="20" t="s">
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>284</v>
       </c>
-      <c r="B19" s="21" t="n">
+      <c r="B19">
         <v>2026</v>
       </c>
-      <c r="C19" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="20" t="s">
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>285</v>
       </c>
-      <c r="B20" s="21" t="n">
+      <c r="B20">
         <v>2026</v>
       </c>
-      <c r="C20" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="20" t="s">
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>286</v>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21">
         <v>2026</v>
       </c>
-      <c r="C21" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="20" t="s">
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>282</v>
       </c>
-      <c r="B22" s="21" t="n">
+      <c r="B22">
         <v>2026</v>
       </c>
-      <c r="C22" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="20" t="s">
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>97</v>
       </c>
-      <c r="B23" s="21" t="n">
+      <c r="B23">
         <v>2026</v>
       </c>
-      <c r="C23" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="20" t="s">
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>287</v>
       </c>
-      <c r="B24" s="21" t="n">
+      <c r="B24">
         <v>2026</v>
       </c>
-      <c r="C24" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="s">
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>288</v>
       </c>
-      <c r="B25" s="21" t="n">
+      <c r="B25">
         <v>2026</v>
       </c>
-      <c r="C25" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="s">
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>278</v>
       </c>
-      <c r="B26" s="21" t="n">
+      <c r="B26">
         <v>2026</v>
       </c>
-      <c r="C26" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="s">
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>289</v>
       </c>
-      <c r="B27" s="21" t="n">
+      <c r="B27">
         <v>2026</v>
       </c>
-      <c r="C27" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="22" t="b">
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added link to latest published paper (PDF) and DOI)
</commit_message>
<xml_diff>
--- a/Data/marsja_publications.xlsx
+++ b/Data/marsja_publications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erima96\Dropbox\BetweenComps\Forskning\CV\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2AD1E030-C0BE-4A48-A096-AF0770B9EDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAFEF7B-4694-4C12-A3FD-E31D5C23F278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,11 @@
     <sheet name="peer_reviews" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="299">
   <si>
     <t>authors</t>
   </si>
@@ -910,13 +909,25 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1Ec9miqeO2wU7uOoXzluMigdVlJJYZLVf/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>10.1044/2026_jslhr-25-01028</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>1-10</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kv_2JQTxy-GMHlXq8YTSwUTRN8K1VDWw/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -925,315 +936,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1241,204 +960,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20 % - Dekorfärg1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Dekorfärg2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Dekorfärg3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Dekorfärg4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Dekorfärg5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Dekorfärg6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Dekorfärg6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Dekorfärg6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Anteckning" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Beräkning" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Bra" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Dekorfärg6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Dålig" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Förklarande text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Indata" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Kontrollcell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Länkad cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Rubrik" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Rubrik 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Rubrik 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Rubrik 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Rubrik 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Summa" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Utdata" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Varningstext" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2374,6 +1907,18 @@
       <c r="D19" t="s">
         <v>116</v>
       </c>
+      <c r="E19" t="s">
+        <v>296</v>
+      </c>
+      <c r="H19" t="s">
+        <v>297</v>
+      </c>
+      <c r="I19" t="s">
+        <v>295</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>298</v>
+      </c>
       <c r="K19" t="b">
         <v>1</v>
       </c>
@@ -2422,10 +1967,13 @@
       <formula1>"accepted,online_first,published"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="J19" r:id="rId1" xr:uid="{F3D89F5F-8BA0-4A7E-98E8-4F5BDC48BB85}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>